<commit_message>
fix: xls background file
</commit_message>
<xml_diff>
--- a/button-design-tokens.xlsx
+++ b/button-design-tokens.xlsx
@@ -584,7 +584,7 @@
   <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -633,7 +633,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>button.bg.primary</t>
+          <t>button.background.primary</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -663,14 +663,14 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Button bg — Primary</t>
+          <t>Button background — Primary</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>button.bg.primary.hover</t>
+          <t>button.background.primary.hover</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -700,14 +700,14 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Button bg — Primary, hover state</t>
+          <t>Button background — Primary, hover state</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>button.bg.primary.active</t>
+          <t>button.background.primary.active</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -737,14 +737,14 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Button bg — Primary, active state</t>
+          <t>Button background — Primary, active state</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>button.bg.primary.disabled</t>
+          <t>button.background.primary.disabled</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -774,14 +774,14 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Button bg — Primary, disabled state</t>
+          <t>Button background — Primary, disabled state</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>button.bg.primary.focus</t>
+          <t>button.background.primary.focus</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Button bg — Primary, focus state</t>
+          <t>Button background — Primary, focus state</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>button.bg.secondary</t>
+          <t>button.background.secondary</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1551,14 +1551,14 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Button bg — Secondary</t>
+          <t>Button background — Secondary</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>button.bg.secondary.hover</t>
+          <t>button.background.secondary.hover</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1588,14 +1588,14 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Button bg — Secondary, hover state</t>
+          <t>Button background — Secondary, hover state</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>button.bg.secondary.active</t>
+          <t>button.background.secondary.active</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -1625,14 +1625,14 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Button bg — Secondary, active state</t>
+          <t>Button background — Secondary, active state</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>button.bg.secondary.disabled</t>
+          <t>button.background.secondary.disabled</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1662,14 +1662,14 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Button bg — Secondary, disabled state</t>
+          <t>Button background — Secondary, disabled state</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>button.bg.secondary.focus</t>
+          <t>button.background.secondary.focus</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Button bg — Secondary, focus state</t>
+          <t>Button background — Secondary, focus state</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>button.bg.cta</t>
+          <t>button.background.cta</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2439,14 +2439,14 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Button bg — CTA</t>
+          <t>Button background — CTA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>button.bg.cta.hover</t>
+          <t>button.background.cta.hover</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2476,14 +2476,14 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Button bg — CTA, hover state</t>
+          <t>Button background — CTA, hover state</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>button.bg.cta.active</t>
+          <t>button.background.cta.active</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -2513,14 +2513,14 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Button bg — CTA, active state</t>
+          <t>Button background — CTA, active state</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>button.bg.cta.disabled</t>
+          <t>button.background.cta.disabled</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2550,14 +2550,14 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Button bg — CTA, disabled state</t>
+          <t>Button background — CTA, disabled state</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>button.bg.cta.focus</t>
+          <t>button.background.cta.focus</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Button bg — CTA, focus state</t>
+          <t>Button background — CTA, focus state</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>button.bg.destructive</t>
+          <t>button.background.destructive</t>
         </is>
       </c>
       <c r="B74" s="9" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -3327,14 +3327,14 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Button bg — Destructive</t>
+          <t>Button background — Destructive</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>button.bg.destructive.hover</t>
+          <t>button.background.destructive.hover</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -3364,14 +3364,14 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Button bg — Destructive, hover state</t>
+          <t>Button background — Destructive, hover state</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>button.bg.destructive.active</t>
+          <t>button.background.destructive.active</t>
         </is>
       </c>
       <c r="B76" s="9" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -3401,14 +3401,14 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Button bg — Destructive, active state</t>
+          <t>Button background — Destructive, active state</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>button.bg.destructive.disabled</t>
+          <t>button.background.destructive.disabled</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -3438,14 +3438,14 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Button bg — Destructive, disabled state</t>
+          <t>Button background — Destructive, disabled state</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>button.bg.destructive.focus</t>
+          <t>button.background.destructive.focus</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Button bg — Destructive, focus state</t>
+          <t>Button background — Destructive, focus state</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4185,7 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>button.bg.highContrast</t>
+          <t>button.background.highContrast</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
@@ -4215,14 +4215,14 @@
       </c>
       <c r="G98" s="11" t="inlineStr">
         <is>
-          <t>Button bg — High-Contrast</t>
+          <t>Button background — High-Contrast</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>button.bg.highContrast.hover</t>
+          <t>button.background.highContrast.hover</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
@@ -4252,14 +4252,14 @@
       </c>
       <c r="G99" s="11" t="inlineStr">
         <is>
-          <t>Button bg — High-Contrast, hover state</t>
+          <t>Button background — High-Contrast, hover state</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>button.bg.highContrast.active</t>
+          <t>button.background.highContrast.active</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
@@ -4289,14 +4289,14 @@
       </c>
       <c r="G100" s="11" t="inlineStr">
         <is>
-          <t>Button bg — High-Contrast, active state</t>
+          <t>Button background — High-Contrast, active state</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>button.bg.highContrast.disabled</t>
+          <t>button.background.highContrast.disabled</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
@@ -4326,14 +4326,14 @@
       </c>
       <c r="G101" s="11" t="inlineStr">
         <is>
-          <t>Button bg — High-Contrast, disabled state</t>
+          <t>Button background — High-Contrast, disabled state</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>button.bg.highContrast.focus</t>
+          <t>button.background.highContrast.focus</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Bg</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="G102" s="11" t="inlineStr">
         <is>
-          <t>Button bg — High-Contrast, focus state</t>
+          <t>Button background — High-Contrast, focus state</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>bg</t>
+          <t>background</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="B26" s="30" t="inlineStr">
         <is>
-          <t>Color elements (bg, text, border, icon)</t>
+          <t>Color elements (background, text, border, icon)</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">

</xml_diff>